<commit_message>
Publish IG build from TeamCity (47)
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-BankAccountNumber1.xlsx
+++ b/docs/StructureDefinition-BankAccountNumber1.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://dips.no/fhir/R4/StructureDefinition/BankAccountNumber1</t>
+    <t>http://DIPS.no/fhir/StructureDefinition/R4/Organization-bankAccountNumber1</t>
   </si>
   <si>
     <t>Version</t>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-03T11:16:58+00:00</t>
+    <t>2026-09-08T11:30:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>